<commit_message>
Update test results: all 50 test cases now show FAIL status
</commit_message>
<xml_diff>
--- a/IT23827080_Assignment 1 - Test cases.xlsx
+++ b/IT23827080_Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Y3S1\ITP M\Assignment\IT23827080\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Y3S1\ITP M\Assignment\IT23827080\IT23827080_Playwright_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53FFA8B-C7C3-42BB-87A0-46078C128024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_7D51F9DD961113450246A35428774AEA525DE7FC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="220">
   <si>
     <t>TC ID</t>
   </si>
@@ -58,9 +58,6 @@
     <t>ඔයාගේ නම මොකක්ද කියලා මට කියන්න පුළුවන්ද?</t>
   </si>
   <si>
-    <t>කොමන්ඩ් ෆෝර්ම්ස්</t>
-  </si>
-  <si>
     <t>FAIL</t>
   </si>
   <si>
@@ -85,21 +82,18 @@
     <t>සුභ අලුත් අවුරුද්දක් වේවා යාලුවනේ!</t>
   </si>
   <si>
+    <t>Greetings</t>
+  </si>
+  <si>
+    <t>It is a standard greeting wishing for the new year</t>
+  </si>
+  <si>
+    <t>It is a standard greeting using Ayubowan</t>
+  </si>
+  <si>
     <t>Requests</t>
   </si>
   <si>
-    <t>UI Error</t>
-  </si>
-  <si>
-    <t>Greetings</t>
-  </si>
-  <si>
-    <t>It is a standard greeting wishing for the new year</t>
-  </si>
-  <si>
-    <t>It is a standard greeting using Ayubowan</t>
-  </si>
-  <si>
     <t>It is a polite request asking for help</t>
   </si>
   <si>
@@ -145,9 +139,6 @@
     <t>ඉක්මන් ඉක්මනට එන්න</t>
   </si>
   <si>
-    <t>රෙපන්ස්</t>
-  </si>
-  <si>
     <t>Repeated Words</t>
   </si>
   <si>
@@ -190,9 +181,6 @@
     <t>මොකක්?? ඒක වෙන්න බැහැ...</t>
   </si>
   <si>
-    <t>ඉන්පුට්ස් with Punctuation Marks</t>
-  </si>
-  <si>
     <t>It uses multiple punctuation marks like ?? and ...</t>
   </si>
   <si>
@@ -220,9 +208,6 @@
     <t>අපි අපේ වැඩක් කරන් ඉඳිමු</t>
   </si>
   <si>
-    <t>රෝමාණිකරණය / ස්පීලිංගේ විකෘති</t>
-  </si>
-  <si>
     <t>The word 'apee' is a spelling variant of 'ape'</t>
   </si>
   <si>
@@ -397,6 +382,9 @@
     <t>අපි Nuwara Eliya trip එකක් යමු</t>
   </si>
   <si>
+    <t>ඩොක් හම්බ වෙන්න යන්න ඕනේ</t>
+  </si>
+  <si>
     <t>Place Names Embedded in Singlish</t>
   </si>
   <si>
@@ -412,6 +400,9 @@
     <t>Kandy වලින් ගන්න පුළුවන්</t>
   </si>
   <si>
+    <t>අපි නුවර එළිය trip එකක් යමු</t>
+  </si>
+  <si>
     <t>Input includes place name 'Kandy'</t>
   </si>
   <si>
@@ -439,6 +430,9 @@
     <t>Nimal සහ sunil meet වෙන්න</t>
   </si>
   <si>
+    <t>නිමල් සහ සුනිල් meet වෙන්න</t>
+  </si>
+  <si>
     <t>Input includes person names 'Nimal' and 'sunil'</t>
   </si>
   <si>
@@ -520,9 +514,6 @@
     <t>අපි 1.00pm ට කතා කරමු</t>
   </si>
   <si>
-    <t>Inputs with Time formats</t>
-  </si>
-  <si>
     <t>Input includes time format '1.00pm'</t>
   </si>
   <si>
@@ -550,7 +541,7 @@
     <t>May 20 වෙනකන් ඉන්න බැහැ</t>
   </si>
   <si>
-    <t>ඉන්පුට්ස් විත් ඩේට්ස්</t>
+    <t>මැයි 20 වෙනකන් ඉන්න බැහැ</t>
   </si>
   <si>
     <t>Input includes date format 'May 20'</t>
@@ -592,9 +583,6 @@
     <t>පට්ට ගති bro ඒක</t>
   </si>
   <si>
-    <t>ඉන්පුට්ස් with Unit of Measurements</t>
-  </si>
-  <si>
     <t>Inputs with Slang and Casual Phrasing</t>
   </si>
   <si>
@@ -610,9 +598,6 @@
     <t>අඩෝ මාර seen එක වුණේ</t>
   </si>
   <si>
-    <t>ඉන්පුට්ස් විත් ස්ලන්ග් and Casual Phrasing</t>
-  </si>
-  <si>
     <t>Input includes slang terms 'ado', 'mara' and 'seen'</t>
   </si>
   <si>
@@ -676,6 +661,9 @@
     <t>oya koheda dan innee?</t>
   </si>
   <si>
+    <t>ඔය කොහෙද දැන් ඉන්නේ?</t>
+  </si>
+  <si>
     <t>ඔයා කොහෙද දැන් ඉන්නේ?</t>
   </si>
   <si>
@@ -688,7 +676,7 @@
     <t>අනේ pls මට කියලා දෙන්නකෝ</t>
   </si>
   <si>
-    <t>question forms</t>
+    <t>අනේ please මට කියලා දෙන්නකෝ</t>
   </si>
   <si>
     <t>It is a polite request</t>
@@ -1121,17 +1109,15 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1142,10 +1128,10 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
         <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1156,10 +1142,10 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1170,36 +1156,34 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
         <v>16</v>
-      </c>
-      <c r="H5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="H6" t="s">
         <v>21</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1210,10 +1194,10 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1224,10 +1208,10 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1238,1012 +1222,1000 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" t="s">
+      <c r="H10" t="s">
         <v>30</v>
-      </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" t="s">
         <v>35</v>
-      </c>
-      <c r="D11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
         <v>39</v>
       </c>
-      <c r="D12" t="s">
+      <c r="H12" t="s">
         <v>40</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" t="s">
-        <v>42</v>
-      </c>
-      <c r="H12" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" t="s">
         <v>44</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>42</v>
-      </c>
-      <c r="H13" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" t="s">
+        <v>48</v>
+      </c>
+      <c r="H14" t="s">
         <v>49</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="F14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" t="s">
-        <v>51</v>
-      </c>
-      <c r="H14" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H15" t="s">
         <v>53</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" t="s">
-        <v>51</v>
-      </c>
-      <c r="H15" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>57</v>
+      </c>
+      <c r="H16" t="s">
         <v>58</v>
-      </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
-      </c>
-      <c r="E17" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G17" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H17" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F18" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G19" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" t="s">
         <v>71</v>
-      </c>
-      <c r="H19" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G20" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H20" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" t="s">
         <v>80</v>
-      </c>
-      <c r="H21" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G22" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="H22" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D23" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G23" t="s">
+        <v>84</v>
+      </c>
+      <c r="H23" t="s">
         <v>89</v>
-      </c>
-      <c r="H23" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H24" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D25" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G25" t="s">
+        <v>93</v>
+      </c>
+      <c r="H25" t="s">
         <v>98</v>
-      </c>
-      <c r="H25" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G26" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H26" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D27" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G27" t="s">
+        <v>102</v>
+      </c>
+      <c r="H27" t="s">
         <v>107</v>
-      </c>
-      <c r="H27" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D28" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G28" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H28" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D29" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G29" t="s">
+        <v>111</v>
+      </c>
+      <c r="H29" t="s">
         <v>116</v>
-      </c>
-      <c r="H29" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D30" t="s">
-        <v>124</v>
+        <v>119</v>
+      </c>
+      <c r="E30" t="s">
+        <v>120</v>
       </c>
       <c r="F30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G30" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H30" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" t="s">
+        <v>125</v>
+      </c>
+      <c r="E31" t="s">
+        <v>126</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
+        <v>121</v>
+      </c>
+      <c r="H31" t="s">
         <v>127</v>
-      </c>
-      <c r="B31" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" t="s">
-        <v>128</v>
-      </c>
-      <c r="D31" t="s">
-        <v>129</v>
-      </c>
-      <c r="F31" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" t="s">
-        <v>125</v>
-      </c>
-      <c r="H31" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" t="s">
+        <v>129</v>
+      </c>
+      <c r="D32" t="s">
+        <v>130</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" t="s">
         <v>131</v>
       </c>
-      <c r="B32" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="H32" t="s">
         <v>132</v>
-      </c>
-      <c r="D32" t="s">
-        <v>133</v>
-      </c>
-      <c r="F32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" t="s">
-        <v>134</v>
-      </c>
-      <c r="H32" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" t="s">
         <v>136</v>
       </c>
-      <c r="B33" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>131</v>
+      </c>
+      <c r="H33" t="s">
         <v>137</v>
-      </c>
-      <c r="D33" t="s">
-        <v>138</v>
-      </c>
-      <c r="F33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" t="s">
-        <v>134</v>
-      </c>
-      <c r="H33" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>138</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>139</v>
+      </c>
+      <c r="D34" t="s">
         <v>140</v>
       </c>
-      <c r="B34" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" t="s">
         <v>141</v>
       </c>
-      <c r="D34" t="s">
+      <c r="H34" t="s">
         <v>142</v>
-      </c>
-      <c r="F34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" t="s">
-        <v>143</v>
-      </c>
-      <c r="H34" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" t="s">
+        <v>144</v>
+      </c>
+      <c r="D35" t="s">
         <v>145</v>
       </c>
-      <c r="B35" t="s">
-        <v>34</v>
-      </c>
-      <c r="C35" t="s">
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" t="s">
+        <v>141</v>
+      </c>
+      <c r="H35" t="s">
         <v>146</v>
-      </c>
-      <c r="D35" t="s">
-        <v>147</v>
-      </c>
-      <c r="F35" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" t="s">
-        <v>143</v>
-      </c>
-      <c r="H35" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" t="s">
+        <v>148</v>
+      </c>
+      <c r="D36" t="s">
         <v>149</v>
       </c>
-      <c r="B36" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="F36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" t="s">
         <v>150</v>
       </c>
-      <c r="D36" t="s">
+      <c r="H36" t="s">
         <v>151</v>
-      </c>
-      <c r="F36" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" t="s">
-        <v>152</v>
-      </c>
-      <c r="H36" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
       </c>
       <c r="C37" t="s">
+        <v>153</v>
+      </c>
+      <c r="D37" t="s">
+        <v>154</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" t="s">
+        <v>150</v>
+      </c>
+      <c r="H37" t="s">
         <v>155</v>
-      </c>
-      <c r="D37" t="s">
-        <v>156</v>
-      </c>
-      <c r="E37" t="s">
-        <v>152</v>
-      </c>
-      <c r="F37" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" t="s">
-        <v>152</v>
-      </c>
-      <c r="H37" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" t="s">
+        <v>157</v>
+      </c>
+      <c r="D38" t="s">
         <v>158</v>
       </c>
-      <c r="B38" t="s">
-        <v>34</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" t="s">
         <v>159</v>
       </c>
-      <c r="D38" t="s">
+      <c r="H38" t="s">
         <v>160</v>
-      </c>
-      <c r="F38" t="s">
-        <v>22</v>
-      </c>
-      <c r="G38" t="s">
-        <v>161</v>
-      </c>
-      <c r="H38" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
       </c>
       <c r="C39" t="s">
+        <v>162</v>
+      </c>
+      <c r="D39" t="s">
+        <v>163</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" t="s">
+        <v>159</v>
+      </c>
+      <c r="H39" t="s">
         <v>164</v>
-      </c>
-      <c r="D39" t="s">
-        <v>165</v>
-      </c>
-      <c r="E39" t="s">
-        <v>166</v>
-      </c>
-      <c r="F39" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" t="s">
-        <v>161</v>
-      </c>
-      <c r="H39" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" t="s">
+        <v>166</v>
+      </c>
+      <c r="D40" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" t="s">
         <v>168</v>
       </c>
-      <c r="B40" t="s">
-        <v>34</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="H40" t="s">
         <v>169</v>
-      </c>
-      <c r="D40" t="s">
-        <v>170</v>
-      </c>
-      <c r="F40" t="s">
-        <v>22</v>
-      </c>
-      <c r="G40" t="s">
-        <v>171</v>
-      </c>
-      <c r="H40" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
       </c>
       <c r="C41" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" t="s">
+        <v>172</v>
+      </c>
+      <c r="E41" t="s">
+        <v>173</v>
+      </c>
+      <c r="F41" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" t="s">
+        <v>168</v>
+      </c>
+      <c r="H41" t="s">
         <v>174</v>
-      </c>
-      <c r="D41" t="s">
-        <v>175</v>
-      </c>
-      <c r="E41" t="s">
-        <v>176</v>
-      </c>
-      <c r="F41" t="s">
-        <v>13</v>
-      </c>
-      <c r="G41" t="s">
-        <v>171</v>
-      </c>
-      <c r="H41" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>175</v>
+      </c>
+      <c r="B42" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" t="s">
+        <v>176</v>
+      </c>
+      <c r="D42" t="s">
+        <v>177</v>
+      </c>
+      <c r="F42" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" t="s">
         <v>178</v>
       </c>
-      <c r="B42" t="s">
-        <v>34</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="H42" t="s">
         <v>179</v>
-      </c>
-      <c r="D42" t="s">
-        <v>180</v>
-      </c>
-      <c r="F42" t="s">
-        <v>22</v>
-      </c>
-      <c r="G42" t="s">
-        <v>181</v>
-      </c>
-      <c r="H42" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
       </c>
       <c r="C43" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D43" t="s">
-        <v>185</v>
+        <v>182</v>
+      </c>
+      <c r="E43" t="s">
+        <v>177</v>
       </c>
       <c r="F43" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G43" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H43" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" t="s">
+        <v>185</v>
+      </c>
+      <c r="D44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E44" t="s">
+        <v>182</v>
+      </c>
+      <c r="F44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" t="s">
         <v>187</v>
       </c>
-      <c r="B44" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="H44" t="s">
         <v>188</v>
-      </c>
-      <c r="D44" t="s">
-        <v>189</v>
-      </c>
-      <c r="E44" t="s">
-        <v>190</v>
-      </c>
-      <c r="F44" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" t="s">
-        <v>191</v>
-      </c>
-      <c r="H44" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
       </c>
       <c r="C45" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D45" t="s">
-        <v>195</v>
-      </c>
-      <c r="E45" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G45" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H45" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
       </c>
       <c r="C46" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D46" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F46" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G46" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="H46" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D47" t="s">
-        <v>205</v>
-      </c>
-      <c r="E47" t="s">
+        <v>200</v>
+      </c>
+      <c r="F47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" t="s">
+        <v>196</v>
+      </c>
+      <c r="H47" t="s">
         <v>201</v>
-      </c>
-      <c r="F47" t="s">
-        <v>13</v>
-      </c>
-      <c r="G47" t="s">
-        <v>201</v>
-      </c>
-      <c r="H47" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B48" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C48" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D48" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="F48" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G48" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="H48" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B49" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C49" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D49" t="s">
-        <v>214</v>
-      </c>
-      <c r="E49" t="s">
+        <v>209</v>
+      </c>
+      <c r="F49" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" t="s">
+        <v>205</v>
+      </c>
+      <c r="H49" t="s">
         <v>210</v>
-      </c>
-      <c r="F49" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" t="s">
-        <v>210</v>
-      </c>
-      <c r="H49" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B50" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C50" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D50" t="s">
-        <v>218</v>
+        <v>213</v>
+      </c>
+      <c r="E50" t="s">
+        <v>214</v>
       </c>
       <c r="F50" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G50" t="s">
+        <v>13</v>
+      </c>
+      <c r="H50" t="s">
         <v>14</v>
-      </c>
-      <c r="H50" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>215</v>
+      </c>
+      <c r="B51" t="s">
+        <v>32</v>
+      </c>
+      <c r="C51" t="s">
+        <v>216</v>
+      </c>
+      <c r="D51" t="s">
+        <v>217</v>
+      </c>
+      <c r="E51" t="s">
+        <v>218</v>
+      </c>
+      <c r="F51" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" t="s">
+        <v>23</v>
+      </c>
+      <c r="H51" t="s">
         <v>219</v>
-      </c>
-      <c r="B51" t="s">
-        <v>34</v>
-      </c>
-      <c r="C51" t="s">
-        <v>220</v>
-      </c>
-      <c r="D51" t="s">
-        <v>221</v>
-      </c>
-      <c r="E51" t="s">
-        <v>222</v>
-      </c>
-      <c r="F51" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" t="s">
-        <v>21</v>
-      </c>
-      <c r="H51" t="s">
-        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test cases with correct results and add retry script
</commit_message>
<xml_diff>
--- a/IT23827080_Assignment 1 - Test cases.xlsx
+++ b/IT23827080_Assignment 1 - Test cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Y3S1\ITP M\Assignment\IT23827080\IT23827080_Playwright_Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Y3S1\ITP M\Assignment\test_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_7D51F9DD961113450246A35428774AEA525DE7FC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72559885-7D15-447F-B7F7-2EAEE48656AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28935" yWindow="1380" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="258">
   <si>
     <t>TC ID</t>
   </si>
@@ -58,6 +58,9 @@
     <t>ඔයාගේ නම මොකක්ද කියලා මට කියන්න පුළුවන්ද?</t>
   </si>
   <si>
+    <t>ඔයාගේ නම මොකක්ද කියලා මට කියන්න පුළුවන්ද</t>
+  </si>
+  <si>
     <t>FAIL</t>
   </si>
   <si>
@@ -82,6 +85,9 @@
     <t>සුභ අලුත් අවුරුද්දක් වේවා යාලුවනේ!</t>
   </si>
   <si>
+    <t>සුභ අලුත් අවුරුද්දක් වේවා යාලුවනේ</t>
+  </si>
+  <si>
     <t>Greetings</t>
   </si>
   <si>
@@ -109,6 +115,9 @@
     <t>එළ එළ, අපි බලමු ඉදිරියට</t>
   </si>
   <si>
+    <t>එළ එළ, අපි බලමු ඉදිරිය</t>
+  </si>
+  <si>
     <t>Responses</t>
   </si>
   <si>
@@ -127,6 +136,9 @@
     <t>ඔව් ඔව්, මම ඒක කරන්නම්</t>
   </si>
   <si>
+    <t>ඔව් ඔව්, මම ඒක කරන්නම</t>
+  </si>
+  <si>
     <t>It is an affirmative response</t>
   </si>
   <si>
@@ -139,6 +151,9 @@
     <t>ඉක්මන් ඉක්මනට එන්න</t>
   </si>
   <si>
+    <t>ඉක්මන් ඉක්මනට එන්</t>
+  </si>
+  <si>
     <t>Repeated Words</t>
   </si>
   <si>
@@ -154,6 +169,9 @@
     <t>ටිකක් ටිකක් රස්නෙයි</t>
   </si>
   <si>
+    <t>ටිකක් ටිකක් රස්නෙය</t>
+  </si>
+  <si>
     <t>The word tikak is repeated</t>
   </si>
   <si>
@@ -166,6 +184,9 @@
     <t>කට්ටිය කොහෙද ඉන්නේ... අපෙනම් නැහැ!</t>
   </si>
   <si>
+    <t>කට්ටිය කොහෙද ඉන්නේ... අපෙනම් නැහැ</t>
+  </si>
+  <si>
     <t>Inputs with Punctuation Marks</t>
   </si>
   <si>
@@ -181,6 +202,9 @@
     <t>මොකක්?? ඒක වෙන්න බැහැ...</t>
   </si>
   <si>
+    <t>මොකක්?? ඒක වෙන්න බැහැ..</t>
+  </si>
+  <si>
     <t>It uses multiple punctuation marks like ?? and ...</t>
   </si>
   <si>
@@ -193,6 +217,9 @@
     <t>මං ඔයාට ආදරෙයි ගොඩක්</t>
   </si>
   <si>
+    <t>මං ඔයාට ආදරෙයි ගොඩක</t>
+  </si>
+  <si>
     <t>Romanization / Spelling Variants</t>
   </si>
   <si>
@@ -208,6 +235,9 @@
     <t>අපි අපේ වැඩක් කරන් ඉඳිමු</t>
   </si>
   <si>
+    <t>අපි අපේ වැඩක් කරන් ඉඳිම</t>
+  </si>
+  <si>
     <t>The word 'apee' is a spelling variant of 'ape'</t>
   </si>
   <si>
@@ -220,6 +250,9 @@
     <t>මම හෙට morning එකේ එන්නම්</t>
   </si>
   <si>
+    <t>මම හෙට morning එකේ එන්නම</t>
+  </si>
+  <si>
     <t>Isolated English Word Insertions in Singlish</t>
   </si>
   <si>
@@ -235,6 +268,9 @@
     <t>මේ phone එකේ battery නැහැ</t>
   </si>
   <si>
+    <t>මේ phone එකේ battery නැහ</t>
+  </si>
+  <si>
     <t>Single English words 'phone' and 'battery' are inserted</t>
   </si>
   <si>
@@ -247,6 +283,9 @@
     <t>අපි all the best කියලා wish කරමු</t>
   </si>
   <si>
+    <t>අපි all the best කියලා wish කරම</t>
+  </si>
+  <si>
     <t>Multi-Word English Phrases in Singlish</t>
   </si>
   <si>
@@ -262,6 +301,9 @@
     <t>එයාට no idea වගේ ඉන්නේ</t>
   </si>
   <si>
+    <t>එයාට no idea වගේ ඉන්න</t>
+  </si>
+  <si>
     <t>A multi-word English phrase 'no idea' is inserted</t>
   </si>
   <si>
@@ -274,6 +316,9 @@
     <t>ඔයාගේ router එකේ password එක දෙන්නකෝ</t>
   </si>
   <si>
+    <t>ඔයාගේ router එකේ password එක දෙන්නක</t>
+  </si>
+  <si>
     <t>English Digital Terms in Singlish</t>
   </si>
   <si>
@@ -289,6 +334,9 @@
     <t>link එක click කරන්න</t>
   </si>
   <si>
+    <t>link එක click කරන්</t>
+  </si>
+  <si>
     <t>Input includes digital terms like 'link' and 'click'</t>
   </si>
   <si>
@@ -301,6 +349,9 @@
     <t>මට instagram එකෙන් msg එකක් දාන්න</t>
   </si>
   <si>
+    <t>මට instagram එකෙන් msg එකක් දාන්</t>
+  </si>
+  <si>
     <t>Platform/App Names in Singlish</t>
   </si>
   <si>
@@ -316,6 +367,9 @@
     <t>youtube එකේ video එක බැලුවා</t>
   </si>
   <si>
+    <t>youtube එකේ video එක බැලුව</t>
+  </si>
+  <si>
     <t>Input includes platform name 'youtube'</t>
   </si>
   <si>
@@ -328,6 +382,9 @@
     <t>මගේ CV එක ASAP එවන්න</t>
   </si>
   <si>
+    <t>මගේ CV එක ASAP එවන්</t>
+  </si>
+  <si>
     <t>English Abbreviations/Acronyms in Singlish</t>
   </si>
   <si>
@@ -343,6 +400,9 @@
     <t>API එක integrate කරමු</t>
   </si>
   <si>
+    <t>API එක integrate කරම</t>
+  </si>
+  <si>
     <t>Input includes abbreviation 'API'</t>
   </si>
   <si>
@@ -355,6 +415,9 @@
     <t>අපේ uni එකේ lab එක හොඳයි</t>
   </si>
   <si>
+    <t>අපේ uni එකේ lab එක හොඳය</t>
+  </si>
+  <si>
     <t>English Clipped Forms in Singlish</t>
   </si>
   <si>
@@ -370,6 +433,9 @@
     <t>doc හම්බ වෙන්න යන්න ඕනේ</t>
   </si>
   <si>
+    <t>doc හම්බ වෙන්න යන්න ඕන</t>
+  </si>
+  <si>
     <t>Input includes clipped word 'doc'</t>
   </si>
   <si>
@@ -382,7 +448,7 @@
     <t>අපි Nuwara Eliya trip එකක් යමු</t>
   </si>
   <si>
-    <t>ඩොක් හම්බ වෙන්න යන්න ඕනේ</t>
+    <t>අපි Nuwara Eliya trip එකක් යම</t>
   </si>
   <si>
     <t>Place Names Embedded in Singlish</t>
@@ -400,7 +466,7 @@
     <t>Kandy වලින් ගන්න පුළුවන්</t>
   </si>
   <si>
-    <t>අපි නුවර එළිය trip එකක් යමු</t>
+    <t>Kandy වලින් ගන්න පුළුවන</t>
   </si>
   <si>
     <t>Input includes place name 'Kandy'</t>
@@ -415,6 +481,9 @@
     <t>Kamal අයියාගේ වැඩ ඉවරද?</t>
   </si>
   <si>
+    <t>Kamal අයියාගේ වැඩ ඉවරද</t>
+  </si>
+  <si>
     <t>Person Names Embedded in Singlish</t>
   </si>
   <si>
@@ -430,7 +499,7 @@
     <t>Nimal සහ sunil meet වෙන්න</t>
   </si>
   <si>
-    <t>නිමල් සහ සුනිල් meet වෙන්න</t>
+    <t>Nimal සහ sunil meet වෙන්</t>
   </si>
   <si>
     <t>Input includes person names 'Nimal' and 'sunil'</t>
@@ -445,6 +514,9 @@
     <t>ළමයි 5දෙනෙක්ම pass වෙලා</t>
   </si>
   <si>
+    <t>ළමයි 5දෙනෙක්ම pass වෙල</t>
+  </si>
+  <si>
     <t>Inputs with Numbers and Numeric Suffixes</t>
   </si>
   <si>
@@ -460,6 +532,9 @@
     <t>2nd එක මගේ</t>
   </si>
   <si>
+    <t>2nd එක මග</t>
+  </si>
+  <si>
     <t>Input includes number with suffix '2nd'</t>
   </si>
   <si>
@@ -472,6 +547,9 @@
     <t>LKR 500ක් විතර යයි</t>
   </si>
   <si>
+    <t>LKR 500ක් විතර යය</t>
+  </si>
+  <si>
     <t>Inputs with Currency</t>
   </si>
   <si>
@@ -487,6 +565,9 @@
     <t>Rs. 25000 පඩියක් ගන්නවා</t>
   </si>
   <si>
+    <t>Rs. 25000 පඩියක් ගන්නව</t>
+  </si>
+  <si>
     <t>Input includes currency 'Rs.'</t>
   </si>
   <si>
@@ -499,6 +580,9 @@
     <t>හෙට 10:30am වෙද්දී එන්න</t>
   </si>
   <si>
+    <t>හෙට 10:30am වෙද්දී එන්</t>
+  </si>
+  <si>
     <t>Inputs with Time Formats</t>
   </si>
   <si>
@@ -514,6 +598,9 @@
     <t>අපි 1.00pm ට කතා කරමු</t>
   </si>
   <si>
+    <t>අපි 1.00pm ට කතා කරම</t>
+  </si>
+  <si>
     <t>Input includes time format '1.00pm'</t>
   </si>
   <si>
@@ -526,6 +613,9 @@
     <t>2024-05-12 වෙනිදා අපි යමු</t>
   </si>
   <si>
+    <t>2024-05-12 වෙනිදා අපි යම</t>
+  </si>
+  <si>
     <t>Inputs with Dates</t>
   </si>
   <si>
@@ -541,7 +631,7 @@
     <t>May 20 වෙනකන් ඉන්න බැහැ</t>
   </si>
   <si>
-    <t>මැයි 20 වෙනකන් ඉන්න බැහැ</t>
+    <t>May 20 වෙනකන් ඉන්න බැහ</t>
   </si>
   <si>
     <t>Input includes date format 'May 20'</t>
@@ -556,6 +646,9 @@
     <t>ඒක 500g ක් ගන්න</t>
   </si>
   <si>
+    <t>ඒක 500g ක් ගන්</t>
+  </si>
+  <si>
     <t>Inputs with Unit of Measurements</t>
   </si>
   <si>
@@ -571,6 +664,9 @@
     <t>3km විතර දුර තියෙනවා</t>
   </si>
   <si>
+    <t>3km විතර දුර තියෙනව</t>
+  </si>
+  <si>
     <t>Input includes unit of measurement 'km'</t>
   </si>
   <si>
@@ -583,6 +679,9 @@
     <t>පට්ට ගති bro ඒක</t>
   </si>
   <si>
+    <t>පට්ට ගති bro ඒ</t>
+  </si>
+  <si>
     <t>Inputs with Slang and Casual Phrasing</t>
   </si>
   <si>
@@ -598,6 +697,9 @@
     <t>අඩෝ මාර seen එක වුණේ</t>
   </si>
   <si>
+    <t>අඩෝ මාර seen එක වුණ</t>
+  </si>
+  <si>
     <t>Input includes slang terms 'ado', 'mara' and 'seen'</t>
   </si>
   <si>
@@ -610,6 +712,9 @@
     <t>මගේ email එක test@gmail.com</t>
   </si>
   <si>
+    <t>මගේ email එක test@gmail.co</t>
+  </si>
+  <si>
     <t>Online Indentifiers in Singlish</t>
   </si>
   <si>
@@ -625,6 +730,9 @@
     <t>https://google.com බලන්න</t>
   </si>
   <si>
+    <t>https://google.com බලන්</t>
+  </si>
+  <si>
     <t>Input includes a URL</t>
   </si>
   <si>
@@ -637,6 +745,9 @@
     <t>මරු කතාව 😂</t>
   </si>
   <si>
+    <t xml:space="preserve">මරු කතාව </t>
+  </si>
+  <si>
     <t>Inputs Containing Emojis</t>
   </si>
   <si>
@@ -652,6 +763,9 @@
     <t>මට ගොඩක් දුකයි 😢</t>
   </si>
   <si>
+    <t xml:space="preserve">මට ගොඩක් දුකයි </t>
+  </si>
+  <si>
     <t>Input includes an emoji 😢</t>
   </si>
   <si>
@@ -661,12 +775,12 @@
     <t>oya koheda dan innee?</t>
   </si>
   <si>
-    <t>ඔය කොහෙද දැන් ඉන්නේ?</t>
-  </si>
-  <si>
     <t>ඔයා කොහෙද දැන් ඉන්නේ?</t>
   </si>
   <si>
+    <t>ඔයා කොහෙද දැන් ඉන්නේ</t>
+  </si>
+  <si>
     <t>Neg_0050</t>
   </si>
   <si>
@@ -676,7 +790,7 @@
     <t>අනේ pls මට කියලා දෙන්නකෝ</t>
   </si>
   <si>
-    <t>අනේ please මට කියලා දෙන්නකෝ</t>
+    <t>අනේ pls මට කියලා දෙන්නක</t>
   </si>
   <si>
     <t>It is a polite request</t>
@@ -1060,14 +1174,14 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.796875" customWidth="1"/>
-    <col min="2" max="2" width="19.19921875" customWidth="1"/>
-    <col min="3" max="3" width="49.69921875" customWidth="1"/>
-    <col min="4" max="4" width="63.796875" customWidth="1"/>
-    <col min="5" max="5" width="38.8984375" customWidth="1"/>
-    <col min="6" max="6" width="18.296875" customWidth="1"/>
-    <col min="7" max="7" width="43.69921875" customWidth="1"/>
-    <col min="8" max="8" width="51.59765625" customWidth="1"/>
+    <col min="1" max="1" width="27.69921875" customWidth="1"/>
+    <col min="2" max="2" width="24.09765625" customWidth="1"/>
+    <col min="3" max="3" width="52.69921875" customWidth="1"/>
+    <col min="4" max="4" width="52.59765625" customWidth="1"/>
+    <col min="5" max="5" width="44.296875" customWidth="1"/>
+    <col min="6" max="6" width="13.796875" customWidth="1"/>
+    <col min="7" max="7" width="48.19921875" customWidth="1"/>
+    <col min="8" max="8" width="49.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1109,15 +1223,17 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1128,10 +1244,10 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1142,10 +1258,10 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1156,34 +1272,36 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="1"/>
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="F6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1194,10 +1312,10 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1208,10 +1326,10 @@
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1222,1000 +1340,1102 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" t="s">
-        <v>29</v>
-      </c>
       <c r="H11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>48</v>
+      </c>
+      <c r="E13" t="s">
+        <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H13" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G14" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H14" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>59</v>
+      </c>
+      <c r="E15" t="s">
+        <v>60</v>
       </c>
       <c r="F15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G15" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H15" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G16" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="H16" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>61</v>
+        <v>70</v>
+      </c>
+      <c r="E17" t="s">
+        <v>71</v>
       </c>
       <c r="F17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G17" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>65</v>
+        <v>75</v>
+      </c>
+      <c r="E18" t="s">
+        <v>76</v>
       </c>
       <c r="F18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>81</v>
+      </c>
+      <c r="E19" t="s">
+        <v>82</v>
       </c>
       <c r="F19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="H19" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>86</v>
+      </c>
+      <c r="E20" t="s">
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G20" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="H20" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>92</v>
+      </c>
+      <c r="E21" t="s">
+        <v>93</v>
       </c>
       <c r="F21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G21" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="H21" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="D22" t="s">
-        <v>83</v>
+        <v>97</v>
+      </c>
+      <c r="E22" t="s">
+        <v>98</v>
       </c>
       <c r="F22" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G22" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="H22" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D23" t="s">
-        <v>88</v>
+        <v>103</v>
+      </c>
+      <c r="E23" t="s">
+        <v>104</v>
       </c>
       <c r="F23" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G23" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="H23" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="D24" t="s">
-        <v>92</v>
+        <v>108</v>
+      </c>
+      <c r="E24" t="s">
+        <v>109</v>
       </c>
       <c r="F24" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G24" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="H24" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="D25" t="s">
-        <v>97</v>
+        <v>114</v>
+      </c>
+      <c r="E25" t="s">
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G25" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="H25" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>119</v>
+      </c>
+      <c r="E26" t="s">
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G26" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="H26" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
-        <v>106</v>
+        <v>125</v>
+      </c>
+      <c r="E27" t="s">
+        <v>126</v>
       </c>
       <c r="F27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G27" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="H27" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C28" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="D28" t="s">
-        <v>110</v>
+        <v>130</v>
+      </c>
+      <c r="E28" t="s">
+        <v>131</v>
       </c>
       <c r="F28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G28" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="H28" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="D29" t="s">
-        <v>115</v>
+        <v>136</v>
+      </c>
+      <c r="E29" t="s">
+        <v>137</v>
       </c>
       <c r="F29" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G29" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="H29" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="D30" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="E30" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="F30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G30" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="H30" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="D31" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="E31" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="F31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G31" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="H31" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="D32" t="s">
-        <v>130</v>
+        <v>152</v>
+      </c>
+      <c r="E32" t="s">
+        <v>153</v>
       </c>
       <c r="F32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G32" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="H32" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C33" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="D33" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="E33" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="F33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G33" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="H33" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C34" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="D34" t="s">
-        <v>140</v>
+        <v>163</v>
+      </c>
+      <c r="E34" t="s">
+        <v>164</v>
       </c>
       <c r="F34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G34" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="H34" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="D35" t="s">
-        <v>145</v>
+        <v>169</v>
+      </c>
+      <c r="E35" t="s">
+        <v>170</v>
       </c>
       <c r="F35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G35" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="H35" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C36" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>149</v>
+        <v>174</v>
+      </c>
+      <c r="E36" t="s">
+        <v>175</v>
       </c>
       <c r="F36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G36" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="H36" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
       </c>
       <c r="C37" t="s">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="D37" t="s">
-        <v>154</v>
+        <v>180</v>
+      </c>
+      <c r="E37" t="s">
+        <v>181</v>
       </c>
       <c r="F37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G37" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="H37" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="B38" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C38" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="D38" t="s">
-        <v>158</v>
+        <v>185</v>
+      </c>
+      <c r="E38" t="s">
+        <v>186</v>
       </c>
       <c r="F38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G38" t="s">
-        <v>159</v>
+        <v>187</v>
       </c>
       <c r="H38" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
       </c>
       <c r="C39" t="s">
-        <v>162</v>
+        <v>190</v>
       </c>
       <c r="D39" t="s">
-        <v>163</v>
+        <v>191</v>
+      </c>
+      <c r="E39" t="s">
+        <v>192</v>
       </c>
       <c r="F39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G39" t="s">
-        <v>159</v>
+        <v>187</v>
       </c>
       <c r="H39" t="s">
-        <v>164</v>
+        <v>193</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>165</v>
+        <v>194</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>166</v>
+        <v>195</v>
       </c>
       <c r="D40" t="s">
-        <v>167</v>
+        <v>196</v>
+      </c>
+      <c r="E40" t="s">
+        <v>197</v>
       </c>
       <c r="F40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G40" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="H40" t="s">
-        <v>169</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
       </c>
       <c r="C41" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="D41" t="s">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="E41" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="F41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G41" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="H41" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>175</v>
+        <v>205</v>
       </c>
       <c r="B42" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C42" t="s">
-        <v>176</v>
+        <v>206</v>
       </c>
       <c r="D42" t="s">
-        <v>177</v>
+        <v>207</v>
+      </c>
+      <c r="E42" t="s">
+        <v>208</v>
       </c>
       <c r="F42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G42" t="s">
-        <v>178</v>
+        <v>209</v>
       </c>
       <c r="H42" t="s">
-        <v>179</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
       </c>
       <c r="C43" t="s">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="D43" t="s">
-        <v>182</v>
+        <v>213</v>
       </c>
       <c r="E43" t="s">
-        <v>177</v>
+        <v>214</v>
       </c>
       <c r="F43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G43" t="s">
-        <v>178</v>
+        <v>209</v>
       </c>
       <c r="H43" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>184</v>
+        <v>216</v>
       </c>
       <c r="B44" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C44" t="s">
-        <v>185</v>
+        <v>217</v>
       </c>
       <c r="D44" t="s">
-        <v>186</v>
+        <v>218</v>
       </c>
       <c r="E44" t="s">
-        <v>182</v>
+        <v>219</v>
       </c>
       <c r="F44" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G44" t="s">
-        <v>187</v>
+        <v>220</v>
       </c>
       <c r="H44" t="s">
-        <v>188</v>
+        <v>221</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>189</v>
+        <v>222</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
       </c>
       <c r="C45" t="s">
-        <v>190</v>
+        <v>223</v>
       </c>
       <c r="D45" t="s">
-        <v>191</v>
+        <v>224</v>
+      </c>
+      <c r="E45" t="s">
+        <v>225</v>
       </c>
       <c r="F45" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G45" t="s">
-        <v>187</v>
+        <v>220</v>
       </c>
       <c r="H45" t="s">
-        <v>192</v>
+        <v>226</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>193</v>
+        <v>227</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
       </c>
       <c r="C46" t="s">
-        <v>194</v>
+        <v>228</v>
       </c>
       <c r="D46" t="s">
-        <v>195</v>
+        <v>229</v>
+      </c>
+      <c r="E46" t="s">
+        <v>230</v>
       </c>
       <c r="F46" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G46" t="s">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="H46" t="s">
-        <v>197</v>
+        <v>232</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>199</v>
+        <v>234</v>
       </c>
       <c r="D47" t="s">
-        <v>200</v>
+        <v>235</v>
+      </c>
+      <c r="E47" t="s">
+        <v>236</v>
       </c>
       <c r="F47" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G47" t="s">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="H47" t="s">
-        <v>201</v>
+        <v>237</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="B48" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C48" t="s">
-        <v>203</v>
+        <v>239</v>
       </c>
       <c r="D48" t="s">
-        <v>204</v>
+        <v>240</v>
+      </c>
+      <c r="E48" t="s">
+        <v>241</v>
       </c>
       <c r="F48" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G48" t="s">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="H48" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>207</v>
+        <v>244</v>
       </c>
       <c r="B49" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C49" t="s">
-        <v>208</v>
+        <v>245</v>
       </c>
       <c r="D49" t="s">
-        <v>209</v>
+        <v>246</v>
+      </c>
+      <c r="E49" t="s">
+        <v>247</v>
       </c>
       <c r="F49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G49" t="s">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="H49" t="s">
-        <v>210</v>
+        <v>248</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>211</v>
+        <v>249</v>
       </c>
       <c r="B50" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C50" t="s">
-        <v>212</v>
+        <v>250</v>
       </c>
       <c r="D50" t="s">
-        <v>213</v>
+        <v>251</v>
       </c>
       <c r="E50" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
       <c r="F50" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H50" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>215</v>
+        <v>253</v>
       </c>
       <c r="B51" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C51" t="s">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="D51" t="s">
-        <v>217</v>
+        <v>255</v>
       </c>
       <c r="E51" t="s">
-        <v>218</v>
+        <v>256</v>
       </c>
       <c r="F51" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G51" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H51" t="s">
-        <v>219</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>